<commit_message>
Upload Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx via attendance app
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Session Analysis Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Analysis Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-15 21:09:32 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-24 15:03:24 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-30 13:00:20 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-30 22:12:54 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-31 12:15:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-06 16:17:37 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-17 16:55:20 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-18 13:00:46 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-20 21:03:39 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-20 22:12:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-21 15:37:04 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-21 17:17:11 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-23 15:49:49 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-24 15:45:52 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-24 18:05:36 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-24 19:55:39 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-24 21:33:07 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-26 07:06:53 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-27 22:13:04 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-27 23:23:22 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-28 15:17:28 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-30 23:23:16 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-05 10:08:27 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-05 13:01:40 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-05 16:00:40 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-05 20:24:34 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-06 20:35:58 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-06 22:07:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-08 16:42:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-10 19:11:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-10 21:45:40 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 05:03:36 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 12:09:08 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 13:22:42 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-14 16:07:22 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-15 00:04:03 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-15 13:00:34 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-16 02:25:09 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-18 04:04:35 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-18 20:17:58 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-19 21:35:23 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-21 00:07:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-22 04:27:36 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-23 06:22:58 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-26 13:25:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-29 01:05:00 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-29 22:38:38 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-01 08:47:50 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-01 12:08:44 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-01 13:54:54 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-03 13:01:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-03 20:51:43 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-05 17:09:33 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-07 10:56:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-08 05:48:03 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 09:43:40 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 18:56:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 20:07:55 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-10 20:00:08 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-11 05:41:16 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-11 17:03:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-12 11:05:44 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-13 08:59:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-13 17:01:18 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>